<commit_message>
Prepare dashboard for cloud deployment
</commit_message>
<xml_diff>
--- a/data/Analytic Code Output/FSM_Child_Coverage_Outreach_Tables_080626.xlsx
+++ b/data/Analytic Code Output/FSM_Child_Coverage_Outreach_Tables_080626.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ikp9\R\USAPI\FSM\FSM_Coverage_Outreach_Dashboard\data\Analytic Code Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F256D7C-6FE1-4E72-9E4C-ADCA6643F7A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD3474B-3C41-4E76-94BB-EBE187214AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,12 @@
     <sheet name="19–35 Mos Coverage by State" sheetId="7" r:id="rId7"/>
     <sheet name="19–35 Mos Series by State" sheetId="8" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'2 – 83 months UTD by County'!$A$3:$E$703</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Undervaccinated by County'!$A$3:$D$563</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Undervaccinated by Village'!$A$3:$D$452</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Vaccines Needed by County'!$A$3:$J$73</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -1463,7 +1469,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1493,20 +1499,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1807,7 +1802,7 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.21875" customWidth="1"/>
     <col min="2" max="6" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2074,10 +2069,10 @@
   <dimension ref="A1:D452"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" customWidth="1"/>
+    <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" customWidth="1"/>
-    <col min="4" max="4" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8389,7 +8384,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D3" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A3:D452" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -8403,7 +8398,7 @@
   <dimension ref="A1:D563"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
     <col min="3" max="3" width="39.5546875" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" customWidth="1"/>
@@ -16272,7 +16267,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D3" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A3:D563" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -16286,18 +16281,18 @@
   <dimension ref="A1:J73"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.77734375" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" customWidth="1"/>
     <col min="5" max="5" width="8.6640625" customWidth="1"/>
     <col min="6" max="6" width="19.6640625" customWidth="1"/>
     <col min="7" max="8" width="18.6640625" customWidth="1"/>
     <col min="9" max="9" width="7.6640625" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>372</v>
       </c>
@@ -16311,7 +16306,7 @@
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
     </row>
-    <row r="3" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>19</v>
       </c>
@@ -18584,7 +18579,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J3" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A3:J73" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -18598,7 +18593,7 @@
   <dimension ref="A1:AU26"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="15" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" customWidth="1"/>
     <col min="3" max="47" width="12.6640625" customWidth="1"/>
   </cols>
@@ -18655,7 +18650,7 @@
       <c r="AU1" s="9"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="10" t="s">
         <v>382</v>
       </c>
       <c r="B2" s="10" t="s">
@@ -18718,7 +18713,7 @@
       <c r="AU2" s="10"/>
     </row>
     <row r="3" spans="1:47" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13"/>
+      <c r="A3" s="10"/>
       <c r="B3" s="10"/>
       <c r="C3" s="1" t="s">
         <v>9</v>
@@ -18857,150 +18852,150 @@
       </c>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>362</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="6">
         <v>68.8</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="6">
         <v>86.1</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="6">
         <v>91</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="6">
         <v>96.1</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="6">
         <v>97.6</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="6">
         <v>98.7</v>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="6">
         <v>99.2</v>
       </c>
-      <c r="J4" s="12">
+      <c r="J4" s="6">
         <v>98.9</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="6">
         <v>98.7</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="6">
         <v>57.6</v>
       </c>
-      <c r="M4" s="12">
+      <c r="M4" s="6">
         <v>78.8</v>
       </c>
-      <c r="N4" s="12">
+      <c r="N4" s="6">
         <v>88</v>
       </c>
-      <c r="O4" s="12">
+      <c r="O4" s="6">
         <v>96.8</v>
       </c>
-      <c r="P4" s="12">
+      <c r="P4" s="6">
         <v>97.7</v>
       </c>
-      <c r="Q4" s="12">
+      <c r="Q4" s="6">
         <v>98.6</v>
       </c>
-      <c r="R4" s="12">
+      <c r="R4" s="6">
         <v>99.2</v>
       </c>
-      <c r="S4" s="12">
+      <c r="S4" s="6">
         <v>99</v>
       </c>
-      <c r="T4" s="12">
+      <c r="T4" s="6">
         <v>98.9</v>
       </c>
-      <c r="U4" s="12">
+      <c r="U4" s="6">
         <v>92.9</v>
       </c>
-      <c r="V4" s="12">
+      <c r="V4" s="6">
         <v>100</v>
       </c>
-      <c r="W4" s="12">
+      <c r="W4" s="6">
         <v>96.2</v>
       </c>
-      <c r="X4" s="12">
+      <c r="X4" s="6">
         <v>100</v>
       </c>
-      <c r="Y4" s="12">
+      <c r="Y4" s="6">
         <v>100</v>
       </c>
-      <c r="Z4" s="12">
+      <c r="Z4" s="6">
         <v>100</v>
       </c>
-      <c r="AA4" s="12">
+      <c r="AA4" s="6">
         <v>99</v>
       </c>
-      <c r="AB4" s="12">
+      <c r="AB4" s="6">
         <v>98</v>
       </c>
-      <c r="AC4" s="12">
+      <c r="AC4" s="6">
         <v>96.7</v>
       </c>
-      <c r="AD4" s="12">
+      <c r="AD4" s="6">
         <v>69.3</v>
       </c>
-      <c r="AE4" s="12">
+      <c r="AE4" s="6">
         <v>87.5</v>
       </c>
-      <c r="AF4" s="12">
+      <c r="AF4" s="6">
         <v>93.1</v>
       </c>
-      <c r="AG4" s="12">
+      <c r="AG4" s="6">
         <v>93.5</v>
       </c>
-      <c r="AH4" s="12">
+      <c r="AH4" s="6">
         <v>96.7</v>
       </c>
-      <c r="AI4" s="12">
+      <c r="AI4" s="6">
         <v>98.2</v>
       </c>
-      <c r="AJ4" s="12">
+      <c r="AJ4" s="6">
         <v>99.1</v>
       </c>
-      <c r="AK4" s="12">
+      <c r="AK4" s="6">
         <v>98.6</v>
       </c>
-      <c r="AL4" s="12">
+      <c r="AL4" s="6">
         <v>98.5</v>
       </c>
-      <c r="AM4" s="12">
+      <c r="AM4" s="6">
         <v>91.7</v>
       </c>
-      <c r="AN4" s="12">
+      <c r="AN4" s="6">
         <v>97.2</v>
       </c>
-      <c r="AO4" s="12">
+      <c r="AO4" s="6">
         <v>94.3</v>
       </c>
-      <c r="AP4" s="12">
+      <c r="AP4" s="6">
         <v>100</v>
       </c>
-      <c r="AQ4" s="12">
+      <c r="AQ4" s="6">
         <v>98.8</v>
       </c>
-      <c r="AR4" s="12">
+      <c r="AR4" s="6">
         <v>100</v>
       </c>
-      <c r="AS4" s="12">
+      <c r="AS4" s="6">
         <v>100</v>
       </c>
-      <c r="AT4" s="12">
+      <c r="AT4" s="6">
         <v>100</v>
       </c>
-      <c r="AU4" s="12">
+      <c r="AU4" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -19009,141 +19004,141 @@
       <c r="C5" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="6">
         <v>49.8</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="6">
         <v>71.5</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="6">
         <v>84.5</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="6">
         <v>91.6</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="6">
         <v>95.7</v>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="6">
         <v>97.3</v>
       </c>
-      <c r="J5" s="12">
+      <c r="J5" s="6">
         <v>97.6</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="6">
         <v>97.2</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="M5" s="12">
+      <c r="M5" s="6">
         <v>40.700000000000003</v>
       </c>
-      <c r="N5" s="12">
+      <c r="N5" s="6">
         <v>61.4</v>
       </c>
-      <c r="O5" s="12">
+      <c r="O5" s="6">
         <v>82.4</v>
       </c>
-      <c r="P5" s="12">
+      <c r="P5" s="6">
         <v>90.2</v>
       </c>
-      <c r="Q5" s="12">
+      <c r="Q5" s="6">
         <v>95.1</v>
       </c>
-      <c r="R5" s="12">
+      <c r="R5" s="6">
         <v>97.2</v>
       </c>
-      <c r="S5" s="12">
+      <c r="S5" s="6">
         <v>97.1</v>
       </c>
-      <c r="T5" s="12">
+      <c r="T5" s="6">
         <v>97.4</v>
       </c>
       <c r="U5" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="V5" s="12">
+      <c r="V5" s="6">
         <v>85</v>
       </c>
-      <c r="W5" s="12">
+      <c r="W5" s="6">
         <v>92.3</v>
       </c>
-      <c r="X5" s="12">
+      <c r="X5" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y5" s="12">
+      <c r="Y5" s="6">
         <v>99.3</v>
       </c>
-      <c r="Z5" s="12">
+      <c r="Z5" s="6">
         <v>100</v>
       </c>
-      <c r="AA5" s="12">
+      <c r="AA5" s="6">
         <v>99</v>
       </c>
-      <c r="AB5" s="12">
+      <c r="AB5" s="6">
         <v>98</v>
       </c>
-      <c r="AC5" s="12">
+      <c r="AC5" s="6">
         <v>96.7</v>
       </c>
       <c r="AD5" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AE5" s="12">
+      <c r="AE5" s="6">
         <v>51.9</v>
       </c>
-      <c r="AF5" s="12">
+      <c r="AF5" s="6">
         <v>77.099999999999994</v>
       </c>
-      <c r="AG5" s="12">
+      <c r="AG5" s="6">
         <v>80.5</v>
       </c>
-      <c r="AH5" s="12">
+      <c r="AH5" s="6">
         <v>90.1</v>
       </c>
-      <c r="AI5" s="12">
+      <c r="AI5" s="6">
         <v>94.5</v>
       </c>
-      <c r="AJ5" s="12">
+      <c r="AJ5" s="6">
         <v>96.5</v>
       </c>
-      <c r="AK5" s="12">
+      <c r="AK5" s="6">
         <v>97.4</v>
       </c>
-      <c r="AL5" s="12">
+      <c r="AL5" s="6">
         <v>96.3</v>
       </c>
       <c r="AM5" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AN5" s="12">
+      <c r="AN5" s="6">
         <v>52.8</v>
       </c>
-      <c r="AO5" s="12">
+      <c r="AO5" s="6">
         <v>83.9</v>
       </c>
-      <c r="AP5" s="12">
+      <c r="AP5" s="6">
         <v>100</v>
       </c>
-      <c r="AQ5" s="12">
+      <c r="AQ5" s="6">
         <v>98.8</v>
       </c>
-      <c r="AR5" s="12">
+      <c r="AR5" s="6">
         <v>100</v>
       </c>
-      <c r="AS5" s="12">
+      <c r="AS5" s="6">
         <v>100</v>
       </c>
-      <c r="AT5" s="12">
+      <c r="AT5" s="6">
         <v>100</v>
       </c>
-      <c r="AU5" s="12">
+      <c r="AU5" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -19155,25 +19150,25 @@
       <c r="D6" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="6">
         <v>45.9</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="6">
         <v>66.3</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="6">
         <v>83.5</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="6">
         <v>90.3</v>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="6">
         <v>94.2</v>
       </c>
-      <c r="J6" s="12">
+      <c r="J6" s="6">
         <v>94.9</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="6">
         <v>95.7</v>
       </c>
       <c r="L6" s="6" t="s">
@@ -19182,25 +19177,25 @@
       <c r="M6" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="N6" s="12">
+      <c r="N6" s="6">
         <v>34.200000000000003</v>
       </c>
-      <c r="O6" s="12">
+      <c r="O6" s="6">
         <v>59.1</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="6">
         <v>81.900000000000006</v>
       </c>
-      <c r="Q6" s="12">
+      <c r="Q6" s="6">
         <v>90</v>
       </c>
-      <c r="R6" s="12">
+      <c r="R6" s="6">
         <v>94.4</v>
       </c>
-      <c r="S6" s="12">
+      <c r="S6" s="6">
         <v>94.7</v>
       </c>
-      <c r="T6" s="12">
+      <c r="T6" s="6">
         <v>96.1</v>
       </c>
       <c r="U6" s="6" t="s">
@@ -19209,25 +19204,25 @@
       <c r="V6" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="W6" s="12">
+      <c r="W6" s="6">
         <v>75</v>
       </c>
-      <c r="X6" s="12">
+      <c r="X6" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y6" s="12">
+      <c r="Y6" s="6">
         <v>98.6</v>
       </c>
-      <c r="Z6" s="12">
+      <c r="Z6" s="6">
         <v>100</v>
       </c>
-      <c r="AA6" s="12">
+      <c r="AA6" s="6">
         <v>98</v>
       </c>
-      <c r="AB6" s="12">
+      <c r="AB6" s="6">
         <v>97</v>
       </c>
-      <c r="AC6" s="12">
+      <c r="AC6" s="6">
         <v>96.7</v>
       </c>
       <c r="AD6" s="6" t="s">
@@ -19236,25 +19231,25 @@
       <c r="AE6" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AF6" s="12">
+      <c r="AF6" s="6">
         <v>51.6</v>
       </c>
-      <c r="AG6" s="12">
+      <c r="AG6" s="6">
         <v>63.7</v>
       </c>
-      <c r="AH6" s="12">
+      <c r="AH6" s="6">
         <v>79</v>
       </c>
-      <c r="AI6" s="12">
+      <c r="AI6" s="6">
         <v>86.3</v>
       </c>
-      <c r="AJ6" s="12">
+      <c r="AJ6" s="6">
         <v>91.6</v>
       </c>
-      <c r="AK6" s="12">
+      <c r="AK6" s="6">
         <v>93.2</v>
       </c>
-      <c r="AL6" s="12">
+      <c r="AL6" s="6">
         <v>93.6</v>
       </c>
       <c r="AM6" s="6" t="s">
@@ -19263,30 +19258,30 @@
       <c r="AN6" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AO6" s="12">
+      <c r="AO6" s="6">
         <v>59.8</v>
       </c>
-      <c r="AP6" s="12">
+      <c r="AP6" s="6">
         <v>89.1</v>
       </c>
-      <c r="AQ6" s="12">
+      <c r="AQ6" s="6">
         <v>98.1</v>
       </c>
-      <c r="AR6" s="12">
+      <c r="AR6" s="6">
         <v>99.5</v>
       </c>
-      <c r="AS6" s="12">
+      <c r="AS6" s="6">
         <v>100</v>
       </c>
-      <c r="AT6" s="12">
+      <c r="AT6" s="6">
         <v>100</v>
       </c>
-      <c r="AU6" s="12">
+      <c r="AU6" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -19301,22 +19296,22 @@
       <c r="E7" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="6">
         <v>25</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="6">
         <v>59.5</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="6">
         <v>78</v>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="6">
         <v>85.8</v>
       </c>
-      <c r="J7" s="12">
+      <c r="J7" s="6">
         <v>89.3</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="6">
         <v>90.6</v>
       </c>
       <c r="L7" s="6" t="s">
@@ -19328,22 +19323,22 @@
       <c r="N7" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="O7" s="12">
+      <c r="O7" s="6">
         <v>15.5</v>
       </c>
-      <c r="P7" s="12">
+      <c r="P7" s="6">
         <v>58</v>
       </c>
-      <c r="Q7" s="12">
+      <c r="Q7" s="6">
         <v>81.2</v>
       </c>
-      <c r="R7" s="12">
+      <c r="R7" s="6">
         <v>86.2</v>
       </c>
-      <c r="S7" s="12">
+      <c r="S7" s="6">
         <v>89.3</v>
       </c>
-      <c r="T7" s="12">
+      <c r="T7" s="6">
         <v>91</v>
       </c>
       <c r="U7" s="6" t="s">
@@ -19355,22 +19350,22 @@
       <c r="W7" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="X7" s="12">
+      <c r="X7" s="6">
         <v>58.5</v>
       </c>
-      <c r="Y7" s="12">
+      <c r="Y7" s="6">
         <v>95.8</v>
       </c>
-      <c r="Z7" s="12">
+      <c r="Z7" s="6">
         <v>100</v>
       </c>
-      <c r="AA7" s="12">
+      <c r="AA7" s="6">
         <v>96</v>
       </c>
-      <c r="AB7" s="12">
+      <c r="AB7" s="6">
         <v>94.9</v>
       </c>
-      <c r="AC7" s="12">
+      <c r="AC7" s="6">
         <v>96.7</v>
       </c>
       <c r="AD7" s="6" t="s">
@@ -19382,22 +19377,22 @@
       <c r="AF7" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AG7" s="12">
+      <c r="AG7" s="6">
         <v>25.2</v>
       </c>
-      <c r="AH7" s="12">
+      <c r="AH7" s="6">
         <v>50</v>
       </c>
-      <c r="AI7" s="12">
+      <c r="AI7" s="6">
         <v>66.900000000000006</v>
       </c>
-      <c r="AJ7" s="12">
+      <c r="AJ7" s="6">
         <v>81.5</v>
       </c>
-      <c r="AK7" s="12">
+      <c r="AK7" s="6">
         <v>84.6</v>
       </c>
-      <c r="AL7" s="12">
+      <c r="AL7" s="6">
         <v>86.5</v>
       </c>
       <c r="AM7" s="6" t="s">
@@ -19409,27 +19404,27 @@
       <c r="AO7" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AP7" s="12">
+      <c r="AP7" s="6">
         <v>47.5</v>
       </c>
-      <c r="AQ7" s="12">
+      <c r="AQ7" s="6">
         <v>79.400000000000006</v>
       </c>
-      <c r="AR7" s="12">
+      <c r="AR7" s="6">
         <v>88</v>
       </c>
-      <c r="AS7" s="12">
+      <c r="AS7" s="6">
         <v>94</v>
       </c>
-      <c r="AT7" s="12">
+      <c r="AT7" s="6">
         <v>99.6</v>
       </c>
-      <c r="AU7" s="12">
+      <c r="AU7" s="6">
         <v>99.5</v>
       </c>
     </row>
     <row r="8" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -19453,13 +19448,13 @@
       <c r="H8" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="6">
         <v>54.1</v>
       </c>
-      <c r="J8" s="12">
+      <c r="J8" s="6">
         <v>80.400000000000006</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="6">
         <v>87.8</v>
       </c>
       <c r="L8" s="6" t="s">
@@ -19480,13 +19475,13 @@
       <c r="Q8" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="R8" s="12">
+      <c r="R8" s="6">
         <v>47.6</v>
       </c>
-      <c r="S8" s="12">
+      <c r="S8" s="6">
         <v>80</v>
       </c>
-      <c r="T8" s="12">
+      <c r="T8" s="6">
         <v>88</v>
       </c>
       <c r="U8" s="6" t="s">
@@ -19507,13 +19502,13 @@
       <c r="Z8" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AA8" s="12">
+      <c r="AA8" s="6">
         <v>54.5</v>
       </c>
-      <c r="AB8" s="12">
+      <c r="AB8" s="6">
         <v>94.9</v>
       </c>
-      <c r="AC8" s="12">
+      <c r="AC8" s="6">
         <v>96.7</v>
       </c>
       <c r="AD8" s="6" t="s">
@@ -19534,13 +19529,13 @@
       <c r="AI8" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AJ8" s="12">
+      <c r="AJ8" s="6">
         <v>59.1</v>
       </c>
-      <c r="AK8" s="12">
+      <c r="AK8" s="6">
         <v>72</v>
       </c>
-      <c r="AL8" s="12">
+      <c r="AL8" s="6">
         <v>82.6</v>
       </c>
       <c r="AM8" s="6" t="s">
@@ -19561,161 +19556,161 @@
       <c r="AR8" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AS8" s="12">
+      <c r="AS8" s="6">
         <v>69</v>
       </c>
-      <c r="AT8" s="12">
+      <c r="AT8" s="6">
         <v>98.7</v>
       </c>
-      <c r="AU8" s="12">
+      <c r="AU8" s="6">
         <v>99.5</v>
       </c>
     </row>
     <row r="9" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="11" t="s">
         <v>363</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="6">
         <v>68.8</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="6">
         <v>86.1</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="6">
         <v>91</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="6">
         <v>96</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="6">
         <v>97.5</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="6">
         <v>98.6</v>
       </c>
-      <c r="I9" s="12">
+      <c r="I9" s="6">
         <v>99.2</v>
       </c>
-      <c r="J9" s="12">
+      <c r="J9" s="6">
         <v>98.9</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="6">
         <v>98.5</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="6">
         <v>57.6</v>
       </c>
-      <c r="M9" s="12">
+      <c r="M9" s="6">
         <v>78.8</v>
       </c>
-      <c r="N9" s="12">
+      <c r="N9" s="6">
         <v>88</v>
       </c>
-      <c r="O9" s="12">
+      <c r="O9" s="6">
         <v>96.5</v>
       </c>
-      <c r="P9" s="12">
+      <c r="P9" s="6">
         <v>97.7</v>
       </c>
-      <c r="Q9" s="12">
+      <c r="Q9" s="6">
         <v>98.5</v>
       </c>
-      <c r="R9" s="12">
+      <c r="R9" s="6">
         <v>99.2</v>
       </c>
-      <c r="S9" s="12">
+      <c r="S9" s="6">
         <v>99</v>
       </c>
-      <c r="T9" s="12">
+      <c r="T9" s="6">
         <v>98.8</v>
       </c>
-      <c r="U9" s="12">
+      <c r="U9" s="6">
         <v>92.9</v>
       </c>
-      <c r="V9" s="12">
+      <c r="V9" s="6">
         <v>100</v>
       </c>
-      <c r="W9" s="12">
+      <c r="W9" s="6">
         <v>96.2</v>
       </c>
-      <c r="X9" s="12">
+      <c r="X9" s="6">
         <v>100</v>
       </c>
-      <c r="Y9" s="12">
+      <c r="Y9" s="6">
         <v>100</v>
       </c>
-      <c r="Z9" s="12">
+      <c r="Z9" s="6">
         <v>100</v>
       </c>
-      <c r="AA9" s="12">
+      <c r="AA9" s="6">
         <v>99</v>
       </c>
-      <c r="AB9" s="12">
+      <c r="AB9" s="6">
         <v>98</v>
       </c>
-      <c r="AC9" s="12">
+      <c r="AC9" s="6">
         <v>96.7</v>
       </c>
-      <c r="AD9" s="12">
+      <c r="AD9" s="6">
         <v>69.3</v>
       </c>
-      <c r="AE9" s="12">
+      <c r="AE9" s="6">
         <v>87.5</v>
       </c>
-      <c r="AF9" s="12">
+      <c r="AF9" s="6">
         <v>93.1</v>
       </c>
-      <c r="AG9" s="12">
+      <c r="AG9" s="6">
         <v>93.5</v>
       </c>
-      <c r="AH9" s="12">
+      <c r="AH9" s="6">
         <v>96.6</v>
       </c>
-      <c r="AI9" s="12">
+      <c r="AI9" s="6">
         <v>98.2</v>
       </c>
-      <c r="AJ9" s="12">
+      <c r="AJ9" s="6">
         <v>99.1</v>
       </c>
-      <c r="AK9" s="12">
+      <c r="AK9" s="6">
         <v>98.6</v>
       </c>
-      <c r="AL9" s="12">
+      <c r="AL9" s="6">
         <v>98.1</v>
       </c>
-      <c r="AM9" s="12">
+      <c r="AM9" s="6">
         <v>91.7</v>
       </c>
-      <c r="AN9" s="12">
+      <c r="AN9" s="6">
         <v>97.2</v>
       </c>
-      <c r="AO9" s="12">
+      <c r="AO9" s="6">
         <v>94.3</v>
       </c>
-      <c r="AP9" s="12">
+      <c r="AP9" s="6">
         <v>100</v>
       </c>
-      <c r="AQ9" s="12">
+      <c r="AQ9" s="6">
         <v>98.8</v>
       </c>
-      <c r="AR9" s="12">
+      <c r="AR9" s="6">
         <v>100</v>
       </c>
-      <c r="AS9" s="12">
+      <c r="AS9" s="6">
         <v>100</v>
       </c>
-      <c r="AT9" s="12">
+      <c r="AT9" s="6">
         <v>100</v>
       </c>
-      <c r="AU9" s="12">
+      <c r="AU9" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -19724,141 +19719,141 @@
       <c r="C10" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="6">
         <v>49.8</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="6">
         <v>71.5</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="6">
         <v>84.4</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="6">
         <v>91.5</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="6">
         <v>95.7</v>
       </c>
-      <c r="I10" s="12">
+      <c r="I10" s="6">
         <v>97.3</v>
       </c>
-      <c r="J10" s="12">
+      <c r="J10" s="6">
         <v>97.5</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="6">
         <v>97.2</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="M10" s="12">
+      <c r="M10" s="6">
         <v>40.700000000000003</v>
       </c>
-      <c r="N10" s="12">
+      <c r="N10" s="6">
         <v>61.4</v>
       </c>
-      <c r="O10" s="12">
+      <c r="O10" s="6">
         <v>82.4</v>
       </c>
-      <c r="P10" s="12">
+      <c r="P10" s="6">
         <v>90.2</v>
       </c>
-      <c r="Q10" s="12">
+      <c r="Q10" s="6">
         <v>95</v>
       </c>
-      <c r="R10" s="12">
+      <c r="R10" s="6">
         <v>97.2</v>
       </c>
-      <c r="S10" s="12">
+      <c r="S10" s="6">
         <v>96.9</v>
       </c>
-      <c r="T10" s="12">
+      <c r="T10" s="6">
         <v>97.4</v>
       </c>
       <c r="U10" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="V10" s="12">
+      <c r="V10" s="6">
         <v>85</v>
       </c>
-      <c r="W10" s="12">
+      <c r="W10" s="6">
         <v>92.3</v>
       </c>
-      <c r="X10" s="12">
+      <c r="X10" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y10" s="12">
+      <c r="Y10" s="6">
         <v>99.3</v>
       </c>
-      <c r="Z10" s="12">
+      <c r="Z10" s="6">
         <v>100</v>
       </c>
-      <c r="AA10" s="12">
+      <c r="AA10" s="6">
         <v>99</v>
       </c>
-      <c r="AB10" s="12">
+      <c r="AB10" s="6">
         <v>98</v>
       </c>
-      <c r="AC10" s="12">
+      <c r="AC10" s="6">
         <v>96.7</v>
       </c>
       <c r="AD10" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AE10" s="12">
+      <c r="AE10" s="6">
         <v>51.9</v>
       </c>
-      <c r="AF10" s="12">
+      <c r="AF10" s="6">
         <v>77.099999999999994</v>
       </c>
-      <c r="AG10" s="12">
+      <c r="AG10" s="6">
         <v>80.2</v>
       </c>
-      <c r="AH10" s="12">
+      <c r="AH10" s="6">
         <v>89.8</v>
       </c>
-      <c r="AI10" s="12">
+      <c r="AI10" s="6">
         <v>94.6</v>
       </c>
-      <c r="AJ10" s="12">
+      <c r="AJ10" s="6">
         <v>96.5</v>
       </c>
-      <c r="AK10" s="12">
+      <c r="AK10" s="6">
         <v>97.4</v>
       </c>
-      <c r="AL10" s="12">
+      <c r="AL10" s="6">
         <v>96.3</v>
       </c>
       <c r="AM10" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AN10" s="12">
+      <c r="AN10" s="6">
         <v>52.8</v>
       </c>
-      <c r="AO10" s="12">
+      <c r="AO10" s="6">
         <v>83.9</v>
       </c>
-      <c r="AP10" s="12">
+      <c r="AP10" s="6">
         <v>100</v>
       </c>
-      <c r="AQ10" s="12">
+      <c r="AQ10" s="6">
         <v>98.8</v>
       </c>
-      <c r="AR10" s="12">
+      <c r="AR10" s="6">
         <v>100</v>
       </c>
-      <c r="AS10" s="12">
+      <c r="AS10" s="6">
         <v>100</v>
       </c>
-      <c r="AT10" s="12">
+      <c r="AT10" s="6">
         <v>100</v>
       </c>
-      <c r="AU10" s="12">
+      <c r="AU10" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -19870,25 +19865,25 @@
       <c r="D11" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="6">
         <v>45.8</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="6">
         <v>66.2</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="6">
         <v>83.3</v>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="6">
         <v>89.9</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="6">
         <v>93.9</v>
       </c>
-      <c r="J11" s="12">
+      <c r="J11" s="6">
         <v>94.6</v>
       </c>
-      <c r="K11" s="12">
+      <c r="K11" s="6">
         <v>95.2</v>
       </c>
       <c r="L11" s="6" t="s">
@@ -19897,25 +19892,25 @@
       <c r="M11" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="6">
         <v>34</v>
       </c>
-      <c r="O11" s="12">
+      <c r="O11" s="6">
         <v>58.9</v>
       </c>
-      <c r="P11" s="12">
+      <c r="P11" s="6">
         <v>81.8</v>
       </c>
-      <c r="Q11" s="12">
+      <c r="Q11" s="6">
         <v>89.4</v>
       </c>
-      <c r="R11" s="12">
+      <c r="R11" s="6">
         <v>94.2</v>
       </c>
-      <c r="S11" s="12">
+      <c r="S11" s="6">
         <v>94</v>
       </c>
-      <c r="T11" s="12">
+      <c r="T11" s="6">
         <v>95.9</v>
       </c>
       <c r="U11" s="6" t="s">
@@ -19924,25 +19919,25 @@
       <c r="V11" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="W11" s="12">
+      <c r="W11" s="6">
         <v>75</v>
       </c>
-      <c r="X11" s="12">
+      <c r="X11" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y11" s="12">
+      <c r="Y11" s="6">
         <v>98.6</v>
       </c>
-      <c r="Z11" s="12">
+      <c r="Z11" s="6">
         <v>100</v>
       </c>
-      <c r="AA11" s="12">
+      <c r="AA11" s="6">
         <v>98</v>
       </c>
-      <c r="AB11" s="12">
+      <c r="AB11" s="6">
         <v>97</v>
       </c>
-      <c r="AC11" s="12">
+      <c r="AC11" s="6">
         <v>96.7</v>
       </c>
       <c r="AD11" s="6" t="s">
@@ -19951,25 +19946,25 @@
       <c r="AE11" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AF11" s="12">
+      <c r="AF11" s="6">
         <v>51.6</v>
       </c>
-      <c r="AG11" s="12">
+      <c r="AG11" s="6">
         <v>63.7</v>
       </c>
-      <c r="AH11" s="12">
+      <c r="AH11" s="6">
         <v>78.5</v>
       </c>
-      <c r="AI11" s="12">
+      <c r="AI11" s="6">
         <v>86</v>
       </c>
-      <c r="AJ11" s="12">
+      <c r="AJ11" s="6">
         <v>91.2</v>
       </c>
-      <c r="AK11" s="12">
+      <c r="AK11" s="6">
         <v>93.2</v>
       </c>
-      <c r="AL11" s="12">
+      <c r="AL11" s="6">
         <v>92.8</v>
       </c>
       <c r="AM11" s="6" t="s">
@@ -19978,30 +19973,30 @@
       <c r="AN11" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AO11" s="12">
+      <c r="AO11" s="6">
         <v>59.8</v>
       </c>
-      <c r="AP11" s="12">
+      <c r="AP11" s="6">
         <v>89.1</v>
       </c>
-      <c r="AQ11" s="12">
+      <c r="AQ11" s="6">
         <v>98.1</v>
       </c>
-      <c r="AR11" s="12">
+      <c r="AR11" s="6">
         <v>99.5</v>
       </c>
-      <c r="AS11" s="12">
+      <c r="AS11" s="6">
         <v>100</v>
       </c>
-      <c r="AT11" s="12">
+      <c r="AT11" s="6">
         <v>100</v>
       </c>
-      <c r="AU11" s="12">
+      <c r="AU11" s="6">
         <v>99.5</v>
       </c>
     </row>
     <row r="12" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -20025,13 +20020,13 @@
       <c r="H12" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="I12" s="12">
+      <c r="I12" s="6">
         <v>56.9</v>
       </c>
-      <c r="J12" s="12">
+      <c r="J12" s="6">
         <v>83.1</v>
       </c>
-      <c r="K12" s="12">
+      <c r="K12" s="6">
         <v>90.5</v>
       </c>
       <c r="L12" s="6" t="s">
@@ -20052,13 +20047,13 @@
       <c r="Q12" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="R12" s="12">
+      <c r="R12" s="6">
         <v>50.7</v>
       </c>
-      <c r="S12" s="12">
+      <c r="S12" s="6">
         <v>82.7</v>
       </c>
-      <c r="T12" s="12">
+      <c r="T12" s="6">
         <v>91.3</v>
       </c>
       <c r="U12" s="6" t="s">
@@ -20079,13 +20074,13 @@
       <c r="Z12" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AA12" s="12">
+      <c r="AA12" s="6">
         <v>57.6</v>
       </c>
-      <c r="AB12" s="12">
+      <c r="AB12" s="6">
         <v>96</v>
       </c>
-      <c r="AC12" s="12">
+      <c r="AC12" s="6">
         <v>95.9</v>
       </c>
       <c r="AD12" s="6" t="s">
@@ -20106,13 +20101,13 @@
       <c r="AI12" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AJ12" s="12">
+      <c r="AJ12" s="6">
         <v>61.6</v>
       </c>
-      <c r="AK12" s="12">
+      <c r="AK12" s="6">
         <v>76.099999999999994</v>
       </c>
-      <c r="AL12" s="12">
+      <c r="AL12" s="6">
         <v>85.9</v>
       </c>
       <c r="AM12" s="6" t="s">
@@ -20133,18 +20128,18 @@
       <c r="AR12" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AS12" s="12">
+      <c r="AS12" s="6">
         <v>70.2</v>
       </c>
-      <c r="AT12" s="12">
+      <c r="AT12" s="6">
         <v>99.1</v>
       </c>
-      <c r="AU12" s="12">
+      <c r="AU12" s="6">
         <v>99.5</v>
       </c>
     </row>
     <row r="13" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="11" t="s">
         <v>364</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -20159,22 +20154,22 @@
       <c r="E13" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="6">
         <v>60.2</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="6">
         <v>86.8</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="6">
         <v>95.1</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="6">
         <v>96.8</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="6">
         <v>97.3</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="6">
         <v>97.3</v>
       </c>
       <c r="L13" s="6" t="s">
@@ -20186,22 +20181,22 @@
       <c r="N13" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="O13" s="12">
+      <c r="O13" s="6">
         <v>55.4</v>
       </c>
-      <c r="P13" s="12">
+      <c r="P13" s="6">
         <v>86.2</v>
       </c>
-      <c r="Q13" s="12">
+      <c r="Q13" s="6">
         <v>94.8</v>
       </c>
-      <c r="R13" s="12">
+      <c r="R13" s="6">
         <v>97</v>
       </c>
-      <c r="S13" s="12">
+      <c r="S13" s="6">
         <v>97.3</v>
       </c>
-      <c r="T13" s="12">
+      <c r="T13" s="6">
         <v>97.8</v>
       </c>
       <c r="U13" s="6" t="s">
@@ -20213,22 +20208,22 @@
       <c r="W13" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="X13" s="12">
+      <c r="X13" s="6">
         <v>66</v>
       </c>
-      <c r="Y13" s="12">
+      <c r="Y13" s="6">
         <v>98.6</v>
       </c>
-      <c r="Z13" s="12">
+      <c r="Z13" s="6">
         <v>100</v>
       </c>
-      <c r="AA13" s="12">
+      <c r="AA13" s="6">
         <v>98</v>
       </c>
-      <c r="AB13" s="12">
+      <c r="AB13" s="6">
         <v>97</v>
       </c>
-      <c r="AC13" s="12">
+      <c r="AC13" s="6">
         <v>96.7</v>
       </c>
       <c r="AD13" s="6" t="s">
@@ -20240,22 +20235,22 @@
       <c r="AF13" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AG13" s="12">
+      <c r="AG13" s="6">
         <v>64.3</v>
       </c>
-      <c r="AH13" s="12">
+      <c r="AH13" s="6">
         <v>83.3</v>
       </c>
-      <c r="AI13" s="12">
+      <c r="AI13" s="6">
         <v>93.3</v>
       </c>
-      <c r="AJ13" s="12">
+      <c r="AJ13" s="6">
         <v>95.4</v>
       </c>
-      <c r="AK13" s="12">
+      <c r="AK13" s="6">
         <v>96.4</v>
       </c>
-      <c r="AL13" s="12">
+      <c r="AL13" s="6">
         <v>96</v>
       </c>
       <c r="AM13" s="6" t="s">
@@ -20267,27 +20262,27 @@
       <c r="AO13" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AP13" s="12">
+      <c r="AP13" s="6">
         <v>63.4</v>
       </c>
-      <c r="AQ13" s="12">
+      <c r="AQ13" s="6">
         <v>94.9</v>
       </c>
-      <c r="AR13" s="12">
+      <c r="AR13" s="6">
         <v>100</v>
       </c>
-      <c r="AS13" s="12">
+      <c r="AS13" s="6">
         <v>100</v>
       </c>
-      <c r="AT13" s="12">
+      <c r="AT13" s="6">
         <v>100</v>
       </c>
-      <c r="AU13" s="12">
+      <c r="AU13" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -20305,19 +20300,19 @@
       <c r="F14" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="6">
         <v>67.5</v>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="6">
         <v>86.6</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="6">
         <v>91.8</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="6">
         <v>92.9</v>
       </c>
-      <c r="K14" s="12">
+      <c r="K14" s="6">
         <v>94.2</v>
       </c>
       <c r="L14" s="6" t="s">
@@ -20332,19 +20327,19 @@
       <c r="O14" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="P14" s="12">
+      <c r="P14" s="6">
         <v>68.400000000000006</v>
       </c>
-      <c r="Q14" s="12">
+      <c r="Q14" s="6">
         <v>88.7</v>
       </c>
-      <c r="R14" s="12">
+      <c r="R14" s="6">
         <v>92.8</v>
       </c>
-      <c r="S14" s="12">
+      <c r="S14" s="6">
         <v>93.8</v>
       </c>
-      <c r="T14" s="12">
+      <c r="T14" s="6">
         <v>95.1</v>
       </c>
       <c r="U14" s="6" t="s">
@@ -20359,19 +20354,19 @@
       <c r="X14" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="Y14" s="12">
+      <c r="Y14" s="6">
         <v>92.4</v>
       </c>
-      <c r="Z14" s="12">
+      <c r="Z14" s="6">
         <v>100</v>
       </c>
-      <c r="AA14" s="12">
+      <c r="AA14" s="6">
         <v>97</v>
       </c>
-      <c r="AB14" s="12">
+      <c r="AB14" s="6">
         <v>96</v>
       </c>
-      <c r="AC14" s="12">
+      <c r="AC14" s="6">
         <v>96.7</v>
       </c>
       <c r="AD14" s="6" t="s">
@@ -20386,19 +20381,19 @@
       <c r="AG14" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AH14" s="12">
+      <c r="AH14" s="6">
         <v>57.2</v>
       </c>
-      <c r="AI14" s="12">
+      <c r="AI14" s="6">
         <v>77.2</v>
       </c>
-      <c r="AJ14" s="12">
+      <c r="AJ14" s="6">
         <v>87.5</v>
       </c>
-      <c r="AK14" s="12">
+      <c r="AK14" s="6">
         <v>89</v>
       </c>
-      <c r="AL14" s="12">
+      <c r="AL14" s="6">
         <v>91</v>
       </c>
       <c r="AM14" s="6" t="s">
@@ -20413,167 +20408,167 @@
       <c r="AP14" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AQ14" s="12">
+      <c r="AQ14" s="6">
         <v>86</v>
       </c>
-      <c r="AR14" s="12">
+      <c r="AR14" s="6">
         <v>100</v>
       </c>
-      <c r="AS14" s="12">
+      <c r="AS14" s="6">
         <v>100</v>
       </c>
-      <c r="AT14" s="12">
+      <c r="AT14" s="6">
         <v>99.6</v>
       </c>
-      <c r="AU14" s="12">
+      <c r="AU14" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="11" t="s">
         <v>365</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="6">
         <v>68.8</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="6">
         <v>86.1</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="6">
         <v>90.8</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="6">
         <v>96</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="6">
         <v>97.5</v>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="6">
         <v>98.6</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="6">
         <v>99.1</v>
       </c>
-      <c r="J15" s="12">
+      <c r="J15" s="6">
         <v>98.5</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="6">
         <v>97.7</v>
       </c>
-      <c r="L15" s="12">
+      <c r="L15" s="6">
         <v>57.6</v>
       </c>
-      <c r="M15" s="12">
+      <c r="M15" s="6">
         <v>78.8</v>
       </c>
-      <c r="N15" s="12">
+      <c r="N15" s="6">
         <v>87.8</v>
       </c>
-      <c r="O15" s="12">
+      <c r="O15" s="6">
         <v>96.5</v>
       </c>
-      <c r="P15" s="12">
+      <c r="P15" s="6">
         <v>97.6</v>
       </c>
-      <c r="Q15" s="12">
+      <c r="Q15" s="6">
         <v>98.5</v>
       </c>
-      <c r="R15" s="12">
+      <c r="R15" s="6">
         <v>99</v>
       </c>
-      <c r="S15" s="12">
+      <c r="S15" s="6">
         <v>98.4</v>
       </c>
-      <c r="T15" s="12">
+      <c r="T15" s="6">
         <v>97.8</v>
       </c>
-      <c r="U15" s="12">
+      <c r="U15" s="6">
         <v>92.9</v>
       </c>
-      <c r="V15" s="12">
+      <c r="V15" s="6">
         <v>100</v>
       </c>
-      <c r="W15" s="12">
+      <c r="W15" s="6">
         <v>96.2</v>
       </c>
-      <c r="X15" s="12">
+      <c r="X15" s="6">
         <v>100</v>
       </c>
-      <c r="Y15" s="12">
+      <c r="Y15" s="6">
         <v>100</v>
       </c>
-      <c r="Z15" s="12">
+      <c r="Z15" s="6">
         <v>100</v>
       </c>
-      <c r="AA15" s="12">
+      <c r="AA15" s="6">
         <v>99</v>
       </c>
-      <c r="AB15" s="12">
+      <c r="AB15" s="6">
         <v>97</v>
       </c>
-      <c r="AC15" s="12">
+      <c r="AC15" s="6">
         <v>96.7</v>
       </c>
-      <c r="AD15" s="12">
+      <c r="AD15" s="6">
         <v>69.3</v>
       </c>
-      <c r="AE15" s="12">
+      <c r="AE15" s="6">
         <v>87.5</v>
       </c>
-      <c r="AF15" s="12">
+      <c r="AF15" s="6">
         <v>92.7</v>
       </c>
-      <c r="AG15" s="12">
+      <c r="AG15" s="6">
         <v>93.5</v>
       </c>
-      <c r="AH15" s="12">
+      <c r="AH15" s="6">
         <v>96.6</v>
       </c>
-      <c r="AI15" s="12">
+      <c r="AI15" s="6">
         <v>98.2</v>
       </c>
-      <c r="AJ15" s="12">
+      <c r="AJ15" s="6">
         <v>99.1</v>
       </c>
-      <c r="AK15" s="12">
+      <c r="AK15" s="6">
         <v>98.3</v>
       </c>
-      <c r="AL15" s="12">
+      <c r="AL15" s="6">
         <v>97.2</v>
       </c>
-      <c r="AM15" s="12">
+      <c r="AM15" s="6">
         <v>91.7</v>
       </c>
-      <c r="AN15" s="12">
+      <c r="AN15" s="6">
         <v>97.2</v>
       </c>
-      <c r="AO15" s="12">
+      <c r="AO15" s="6">
         <v>94.3</v>
       </c>
-      <c r="AP15" s="12">
+      <c r="AP15" s="6">
         <v>100</v>
       </c>
-      <c r="AQ15" s="12">
+      <c r="AQ15" s="6">
         <v>99.2</v>
       </c>
-      <c r="AR15" s="12">
+      <c r="AR15" s="6">
         <v>100</v>
       </c>
-      <c r="AS15" s="12">
+      <c r="AS15" s="6">
         <v>100</v>
       </c>
-      <c r="AT15" s="12">
+      <c r="AT15" s="6">
         <v>100</v>
       </c>
-      <c r="AU15" s="12">
+      <c r="AU15" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -20582,141 +20577,141 @@
       <c r="C16" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="6">
         <v>49.1</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="6">
         <v>70.5</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="6">
         <v>84.1</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="6">
         <v>90.3</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="6">
         <v>92.1</v>
       </c>
-      <c r="I16" s="12">
+      <c r="I16" s="6">
         <v>92.2</v>
       </c>
-      <c r="J16" s="12">
+      <c r="J16" s="6">
         <v>89.8</v>
       </c>
-      <c r="K16" s="12">
+      <c r="K16" s="6">
         <v>90.6</v>
       </c>
       <c r="L16" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="M16" s="12">
+      <c r="M16" s="6">
         <v>38.9</v>
       </c>
-      <c r="N16" s="12">
+      <c r="N16" s="6">
         <v>61.1</v>
       </c>
-      <c r="O16" s="12">
+      <c r="O16" s="6">
         <v>82</v>
       </c>
-      <c r="P16" s="12">
+      <c r="P16" s="6">
         <v>88.2</v>
       </c>
-      <c r="Q16" s="12">
+      <c r="Q16" s="6">
         <v>89.9</v>
       </c>
-      <c r="R16" s="12">
+      <c r="R16" s="6">
         <v>89.5</v>
       </c>
-      <c r="S16" s="12">
+      <c r="S16" s="6">
         <v>85</v>
       </c>
-      <c r="T16" s="12">
+      <c r="T16" s="6">
         <v>88.1</v>
       </c>
       <c r="U16" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="V16" s="12">
+      <c r="V16" s="6">
         <v>85</v>
       </c>
-      <c r="W16" s="12">
+      <c r="W16" s="6">
         <v>88.5</v>
       </c>
-      <c r="X16" s="12">
+      <c r="X16" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y16" s="12">
+      <c r="Y16" s="6">
         <v>99.3</v>
       </c>
-      <c r="Z16" s="12">
+      <c r="Z16" s="6">
         <v>100</v>
       </c>
-      <c r="AA16" s="12">
+      <c r="AA16" s="6">
         <v>97</v>
       </c>
-      <c r="AB16" s="12">
+      <c r="AB16" s="6">
         <v>97</v>
       </c>
-      <c r="AC16" s="12">
+      <c r="AC16" s="6">
         <v>96.7</v>
       </c>
       <c r="AD16" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AE16" s="12">
+      <c r="AE16" s="6">
         <v>51.9</v>
       </c>
-      <c r="AF16" s="12">
+      <c r="AF16" s="6">
         <v>75.3</v>
       </c>
-      <c r="AG16" s="12">
+      <c r="AG16" s="6">
         <v>80.5</v>
       </c>
-      <c r="AH16" s="12">
+      <c r="AH16" s="6">
         <v>89.1</v>
       </c>
-      <c r="AI16" s="12">
+      <c r="AI16" s="6">
         <v>91.5</v>
       </c>
-      <c r="AJ16" s="12">
+      <c r="AJ16" s="6">
         <v>93</v>
       </c>
-      <c r="AK16" s="12">
+      <c r="AK16" s="6">
         <v>91.5</v>
       </c>
-      <c r="AL16" s="12">
+      <c r="AL16" s="6">
         <v>90.2</v>
       </c>
       <c r="AM16" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AN16" s="12">
+      <c r="AN16" s="6">
         <v>52.8</v>
       </c>
-      <c r="AO16" s="12">
+      <c r="AO16" s="6">
         <v>83.9</v>
       </c>
-      <c r="AP16" s="12">
+      <c r="AP16" s="6">
         <v>99</v>
       </c>
-      <c r="AQ16" s="12">
+      <c r="AQ16" s="6">
         <v>98.8</v>
       </c>
-      <c r="AR16" s="12">
+      <c r="AR16" s="6">
         <v>100</v>
       </c>
-      <c r="AS16" s="12">
+      <c r="AS16" s="6">
         <v>100</v>
       </c>
-      <c r="AT16" s="12">
+      <c r="AT16" s="6">
         <v>100</v>
       </c>
-      <c r="AU16" s="12">
+      <c r="AU16" s="6">
         <v>98.6</v>
       </c>
     </row>
     <row r="17" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -20728,25 +20723,25 @@
       <c r="D17" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="6">
         <v>29.4</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="6">
         <v>56.7</v>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="6">
         <v>74.400000000000006</v>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="6">
         <v>74.900000000000006</v>
       </c>
-      <c r="I17" s="12">
+      <c r="I17" s="6">
         <v>77.900000000000006</v>
       </c>
-      <c r="J17" s="12">
+      <c r="J17" s="6">
         <v>74.2</v>
       </c>
-      <c r="K17" s="12">
+      <c r="K17" s="6">
         <v>77.2</v>
       </c>
       <c r="L17" s="6" t="s">
@@ -20755,25 +20750,25 @@
       <c r="M17" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="N17" s="12">
+      <c r="N17" s="6">
         <v>22.6</v>
       </c>
-      <c r="O17" s="12">
+      <c r="O17" s="6">
         <v>51.5</v>
       </c>
-      <c r="P17" s="12">
+      <c r="P17" s="6">
         <v>69.8</v>
       </c>
-      <c r="Q17" s="12">
+      <c r="Q17" s="6">
         <v>68.2</v>
       </c>
-      <c r="R17" s="12">
+      <c r="R17" s="6">
         <v>73.599999999999994</v>
       </c>
-      <c r="S17" s="12">
+      <c r="S17" s="6">
         <v>64.3</v>
       </c>
-      <c r="T17" s="12">
+      <c r="T17" s="6">
         <v>71.900000000000006</v>
       </c>
       <c r="U17" s="6" t="s">
@@ -20782,25 +20777,25 @@
       <c r="V17" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="W17" s="12">
+      <c r="W17" s="6">
         <v>9.6</v>
       </c>
-      <c r="X17" s="12">
+      <c r="X17" s="6">
         <v>66</v>
       </c>
-      <c r="Y17" s="12">
+      <c r="Y17" s="6">
         <v>96.5</v>
       </c>
-      <c r="Z17" s="12">
+      <c r="Z17" s="6">
         <v>100</v>
       </c>
-      <c r="AA17" s="12">
+      <c r="AA17" s="6">
         <v>96</v>
       </c>
-      <c r="AB17" s="12">
+      <c r="AB17" s="6">
         <v>93.9</v>
       </c>
-      <c r="AC17" s="12">
+      <c r="AC17" s="6">
         <v>95.9</v>
       </c>
       <c r="AD17" s="6" t="s">
@@ -20809,25 +20804,25 @@
       <c r="AE17" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AF17" s="12">
+      <c r="AF17" s="6">
         <v>36</v>
       </c>
-      <c r="AG17" s="12">
+      <c r="AG17" s="6">
         <v>55.5</v>
       </c>
-      <c r="AH17" s="12">
+      <c r="AH17" s="6">
         <v>70.400000000000006</v>
       </c>
-      <c r="AI17" s="12">
+      <c r="AI17" s="6">
         <v>72.5</v>
       </c>
-      <c r="AJ17" s="12">
+      <c r="AJ17" s="6">
         <v>75.5</v>
       </c>
-      <c r="AK17" s="12">
+      <c r="AK17" s="6">
         <v>76.099999999999994</v>
       </c>
-      <c r="AL17" s="12">
+      <c r="AL17" s="6">
         <v>75.7</v>
       </c>
       <c r="AM17" s="6" t="s">
@@ -20836,316 +20831,316 @@
       <c r="AN17" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AO17" s="12">
+      <c r="AO17" s="6">
         <v>49.4</v>
       </c>
-      <c r="AP17" s="12">
+      <c r="AP17" s="6">
         <v>78.2</v>
       </c>
-      <c r="AQ17" s="12">
+      <c r="AQ17" s="6">
         <v>95.7</v>
       </c>
-      <c r="AR17" s="12">
+      <c r="AR17" s="6">
         <v>99</v>
       </c>
-      <c r="AS17" s="12">
+      <c r="AS17" s="6">
         <v>98.8</v>
       </c>
-      <c r="AT17" s="12">
+      <c r="AT17" s="6">
         <v>97.8</v>
       </c>
-      <c r="AU17" s="12">
+      <c r="AU17" s="6">
         <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="11" t="s">
         <v>366</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="6">
         <v>98.2</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="6">
         <v>100</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="6">
         <v>99.2</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="6">
         <v>99.6</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="6">
         <v>99.7</v>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="6">
         <v>99.9</v>
       </c>
-      <c r="I18" s="12">
+      <c r="I18" s="6">
         <v>99.8</v>
       </c>
-      <c r="J18" s="12">
+      <c r="J18" s="6">
         <v>99.6</v>
       </c>
-      <c r="K18" s="12">
+      <c r="K18" s="6">
         <v>99</v>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="6">
         <v>96.5</v>
       </c>
-      <c r="M18" s="12">
+      <c r="M18" s="6">
         <v>100</v>
       </c>
-      <c r="N18" s="12">
+      <c r="N18" s="6">
         <v>98.9</v>
       </c>
-      <c r="O18" s="12">
+      <c r="O18" s="6">
         <v>99.1</v>
       </c>
-      <c r="P18" s="12">
+      <c r="P18" s="6">
         <v>99.6</v>
       </c>
-      <c r="Q18" s="12">
+      <c r="Q18" s="6">
         <v>99.8</v>
       </c>
-      <c r="R18" s="12">
+      <c r="R18" s="6">
         <v>99.9</v>
       </c>
-      <c r="S18" s="12">
+      <c r="S18" s="6">
         <v>99.5</v>
       </c>
-      <c r="T18" s="12">
+      <c r="T18" s="6">
         <v>99.2</v>
       </c>
-      <c r="U18" s="12">
+      <c r="U18" s="6">
         <v>100</v>
       </c>
-      <c r="V18" s="12">
+      <c r="V18" s="6">
         <v>100</v>
       </c>
-      <c r="W18" s="12">
+      <c r="W18" s="6">
         <v>100</v>
       </c>
-      <c r="X18" s="12">
+      <c r="X18" s="6">
         <v>100</v>
       </c>
-      <c r="Y18" s="12">
+      <c r="Y18" s="6">
         <v>100</v>
       </c>
-      <c r="Z18" s="12">
+      <c r="Z18" s="6">
         <v>100</v>
       </c>
-      <c r="AA18" s="12">
+      <c r="AA18" s="6">
         <v>99</v>
       </c>
-      <c r="AB18" s="12">
+      <c r="AB18" s="6">
         <v>99</v>
       </c>
-      <c r="AC18" s="12">
+      <c r="AC18" s="6">
         <v>96.7</v>
       </c>
-      <c r="AD18" s="12">
+      <c r="AD18" s="6">
         <v>99</v>
       </c>
-      <c r="AE18" s="12">
+      <c r="AE18" s="6">
         <v>100</v>
       </c>
-      <c r="AF18" s="12">
+      <c r="AF18" s="6">
         <v>99.3</v>
       </c>
-      <c r="AG18" s="12">
+      <c r="AG18" s="6">
         <v>100</v>
       </c>
-      <c r="AH18" s="12">
+      <c r="AH18" s="6">
         <v>99.8</v>
       </c>
-      <c r="AI18" s="12">
+      <c r="AI18" s="6">
         <v>100</v>
       </c>
-      <c r="AJ18" s="12">
+      <c r="AJ18" s="6">
         <v>99.8</v>
       </c>
-      <c r="AK18" s="12">
+      <c r="AK18" s="6">
         <v>99.7</v>
       </c>
-      <c r="AL18" s="12">
+      <c r="AL18" s="6">
         <v>98.8</v>
       </c>
-      <c r="AM18" s="12">
+      <c r="AM18" s="6">
         <v>100</v>
       </c>
-      <c r="AN18" s="12">
+      <c r="AN18" s="6">
         <v>100</v>
       </c>
-      <c r="AO18" s="12">
+      <c r="AO18" s="6">
         <v>100</v>
       </c>
-      <c r="AP18" s="12">
+      <c r="AP18" s="6">
         <v>100</v>
       </c>
-      <c r="AQ18" s="12">
+      <c r="AQ18" s="6">
         <v>100</v>
       </c>
-      <c r="AR18" s="12">
+      <c r="AR18" s="6">
         <v>100</v>
       </c>
-      <c r="AS18" s="12">
+      <c r="AS18" s="6">
         <v>100</v>
       </c>
-      <c r="AT18" s="12">
+      <c r="AT18" s="6">
         <v>100</v>
       </c>
-      <c r="AU18" s="12">
+      <c r="AU18" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="6">
         <v>64.3</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="6">
         <v>78</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="6">
         <v>83.6</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="6">
         <v>91.7</v>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="6">
         <v>95.7</v>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="6">
         <v>97.6</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="6">
         <v>98.6</v>
       </c>
-      <c r="J19" s="12">
+      <c r="J19" s="6">
         <v>98.3</v>
       </c>
-      <c r="K19" s="12">
+      <c r="K19" s="6">
         <v>97.9</v>
       </c>
-      <c r="L19" s="12">
+      <c r="L19" s="6">
         <v>48.2</v>
       </c>
-      <c r="M19" s="12">
+      <c r="M19" s="6">
         <v>61.1</v>
       </c>
-      <c r="N19" s="12">
+      <c r="N19" s="6">
         <v>74.7</v>
       </c>
-      <c r="O19" s="12">
+      <c r="O19" s="6">
         <v>88</v>
       </c>
-      <c r="P19" s="12">
+      <c r="P19" s="6">
         <v>94.4</v>
       </c>
-      <c r="Q19" s="12">
+      <c r="Q19" s="6">
         <v>96.5</v>
       </c>
-      <c r="R19" s="12">
+      <c r="R19" s="6">
         <v>98.3</v>
       </c>
-      <c r="S19" s="12">
+      <c r="S19" s="6">
         <v>97.8</v>
       </c>
-      <c r="T19" s="12">
+      <c r="T19" s="6">
         <v>98</v>
       </c>
-      <c r="U19" s="12">
+      <c r="U19" s="6">
         <v>78.599999999999994</v>
       </c>
-      <c r="V19" s="12">
+      <c r="V19" s="6">
         <v>95</v>
       </c>
-      <c r="W19" s="12">
+      <c r="W19" s="6">
         <v>96.2</v>
       </c>
-      <c r="X19" s="12">
+      <c r="X19" s="6">
         <v>100</v>
       </c>
-      <c r="Y19" s="12">
+      <c r="Y19" s="6">
         <v>100</v>
       </c>
-      <c r="Z19" s="12">
+      <c r="Z19" s="6">
         <v>100</v>
       </c>
-      <c r="AA19" s="12">
+      <c r="AA19" s="6">
         <v>99</v>
       </c>
-      <c r="AB19" s="12">
+      <c r="AB19" s="6">
         <v>98</v>
       </c>
-      <c r="AC19" s="12">
+      <c r="AC19" s="6">
         <v>96.7</v>
       </c>
-      <c r="AD19" s="12">
+      <c r="AD19" s="6">
         <v>69.3</v>
       </c>
-      <c r="AE19" s="12">
+      <c r="AE19" s="6">
         <v>87.5</v>
       </c>
-      <c r="AF19" s="12">
+      <c r="AF19" s="6">
         <v>90.2</v>
       </c>
-      <c r="AG19" s="12">
+      <c r="AG19" s="6">
         <v>92.6</v>
       </c>
-      <c r="AH19" s="12">
+      <c r="AH19" s="6">
         <v>95.8</v>
       </c>
-      <c r="AI19" s="12">
+      <c r="AI19" s="6">
         <v>97.9</v>
       </c>
-      <c r="AJ19" s="12">
+      <c r="AJ19" s="6">
         <v>98.7</v>
       </c>
-      <c r="AK19" s="12">
+      <c r="AK19" s="6">
         <v>98.3</v>
       </c>
-      <c r="AL19" s="12">
+      <c r="AL19" s="6">
         <v>97.4</v>
       </c>
-      <c r="AM19" s="12">
+      <c r="AM19" s="6">
         <v>91.7</v>
       </c>
-      <c r="AN19" s="12">
+      <c r="AN19" s="6">
         <v>94.4</v>
       </c>
-      <c r="AO19" s="12">
+      <c r="AO19" s="6">
         <v>93.1</v>
       </c>
-      <c r="AP19" s="12">
+      <c r="AP19" s="6">
         <v>100</v>
       </c>
-      <c r="AQ19" s="12">
+      <c r="AQ19" s="6">
         <v>98.8</v>
       </c>
-      <c r="AR19" s="12">
+      <c r="AR19" s="6">
         <v>100</v>
       </c>
-      <c r="AS19" s="12">
+      <c r="AS19" s="6">
         <v>100</v>
       </c>
-      <c r="AT19" s="12">
+      <c r="AT19" s="6">
         <v>100</v>
       </c>
-      <c r="AU19" s="12">
+      <c r="AU19" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -21157,25 +21152,25 @@
       <c r="D20" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="6">
         <v>66.8</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="6">
         <v>78.099999999999994</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="6">
         <v>89.2</v>
       </c>
-      <c r="H20" s="12">
+      <c r="H20" s="6">
         <v>94</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="6">
         <v>95.8</v>
       </c>
-      <c r="J20" s="12">
+      <c r="J20" s="6">
         <v>96.6</v>
       </c>
-      <c r="K20" s="12">
+      <c r="K20" s="6">
         <v>96.2</v>
       </c>
       <c r="L20" s="6" t="s">
@@ -21184,25 +21179,25 @@
       <c r="M20" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="N20" s="12">
+      <c r="N20" s="6">
         <v>52.4</v>
       </c>
-      <c r="O20" s="12">
+      <c r="O20" s="6">
         <v>70</v>
       </c>
-      <c r="P20" s="12">
+      <c r="P20" s="6">
         <v>85.7</v>
       </c>
-      <c r="Q20" s="12">
+      <c r="Q20" s="6">
         <v>92</v>
       </c>
-      <c r="R20" s="12">
+      <c r="R20" s="6">
         <v>94.4</v>
       </c>
-      <c r="S20" s="12">
+      <c r="S20" s="6">
         <v>95.1</v>
       </c>
-      <c r="T20" s="12">
+      <c r="T20" s="6">
         <v>96</v>
       </c>
       <c r="U20" s="6" t="s">
@@ -21211,25 +21206,25 @@
       <c r="V20" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="W20" s="12">
+      <c r="W20" s="6">
         <v>92.3</v>
       </c>
-      <c r="X20" s="12">
+      <c r="X20" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y20" s="12">
+      <c r="Y20" s="6">
         <v>98.6</v>
       </c>
-      <c r="Z20" s="12">
+      <c r="Z20" s="6">
         <v>100</v>
       </c>
-      <c r="AA20" s="12">
+      <c r="AA20" s="6">
         <v>98</v>
       </c>
-      <c r="AB20" s="12">
+      <c r="AB20" s="6">
         <v>97</v>
       </c>
-      <c r="AC20" s="12">
+      <c r="AC20" s="6">
         <v>96.7</v>
       </c>
       <c r="AD20" s="6" t="s">
@@ -21238,25 +21233,25 @@
       <c r="AE20" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AF20" s="12">
+      <c r="AF20" s="6">
         <v>76.400000000000006</v>
       </c>
-      <c r="AG20" s="12">
+      <c r="AG20" s="6">
         <v>79.900000000000006</v>
       </c>
-      <c r="AH20" s="12">
+      <c r="AH20" s="6">
         <v>89.4</v>
       </c>
-      <c r="AI20" s="12">
+      <c r="AI20" s="6">
         <v>94</v>
       </c>
-      <c r="AJ20" s="12">
+      <c r="AJ20" s="6">
         <v>96.4</v>
       </c>
-      <c r="AK20" s="12">
+      <c r="AK20" s="6">
         <v>97.2</v>
       </c>
-      <c r="AL20" s="12">
+      <c r="AL20" s="6">
         <v>95.3</v>
       </c>
       <c r="AM20" s="6" t="s">
@@ -21265,173 +21260,173 @@
       <c r="AN20" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AO20" s="12">
+      <c r="AO20" s="6">
         <v>81.599999999999994</v>
       </c>
-      <c r="AP20" s="12">
+      <c r="AP20" s="6">
         <v>96</v>
       </c>
-      <c r="AQ20" s="12">
+      <c r="AQ20" s="6">
         <v>98.4</v>
       </c>
-      <c r="AR20" s="12">
+      <c r="AR20" s="6">
         <v>100</v>
       </c>
-      <c r="AS20" s="12">
+      <c r="AS20" s="6">
         <v>99.4</v>
       </c>
-      <c r="AT20" s="12">
+      <c r="AT20" s="6">
         <v>100</v>
       </c>
-      <c r="AU20" s="12">
+      <c r="AU20" s="6">
         <v>99.5</v>
       </c>
     </row>
     <row r="21" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="11" t="s">
         <v>367</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="6">
         <v>68.8</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="6">
         <v>86.1</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="6">
         <v>90.9</v>
       </c>
-      <c r="F21" s="12">
+      <c r="F21" s="6">
         <v>95.7</v>
       </c>
-      <c r="G21" s="12">
+      <c r="G21" s="6">
         <v>97.5</v>
       </c>
-      <c r="H21" s="12">
+      <c r="H21" s="6">
         <v>98.3</v>
       </c>
-      <c r="I21" s="12">
+      <c r="I21" s="6">
         <v>99.1</v>
       </c>
-      <c r="J21" s="12">
+      <c r="J21" s="6">
         <v>98.3</v>
       </c>
-      <c r="K21" s="12">
+      <c r="K21" s="6">
         <v>97.6</v>
       </c>
-      <c r="L21" s="12">
+      <c r="L21" s="6">
         <v>57.6</v>
       </c>
-      <c r="M21" s="12">
+      <c r="M21" s="6">
         <v>78.8</v>
       </c>
-      <c r="N21" s="12">
+      <c r="N21" s="6">
         <v>87.8</v>
       </c>
-      <c r="O21" s="12">
+      <c r="O21" s="6">
         <v>96.1</v>
       </c>
-      <c r="P21" s="12">
+      <c r="P21" s="6">
         <v>97.5</v>
       </c>
-      <c r="Q21" s="12">
+      <c r="Q21" s="6">
         <v>98</v>
       </c>
-      <c r="R21" s="12">
+      <c r="R21" s="6">
         <v>99</v>
       </c>
-      <c r="S21" s="12">
+      <c r="S21" s="6">
         <v>98.4</v>
       </c>
-      <c r="T21" s="12">
+      <c r="T21" s="6">
         <v>97.6</v>
       </c>
-      <c r="U21" s="12">
+      <c r="U21" s="6">
         <v>92.9</v>
       </c>
-      <c r="V21" s="12">
+      <c r="V21" s="6">
         <v>100</v>
       </c>
-      <c r="W21" s="12">
+      <c r="W21" s="6">
         <v>96.2</v>
       </c>
-      <c r="X21" s="12">
+      <c r="X21" s="6">
         <v>100</v>
       </c>
-      <c r="Y21" s="12">
+      <c r="Y21" s="6">
         <v>100</v>
       </c>
-      <c r="Z21" s="12">
+      <c r="Z21" s="6">
         <v>100</v>
       </c>
-      <c r="AA21" s="12">
+      <c r="AA21" s="6">
         <v>99</v>
       </c>
-      <c r="AB21" s="12">
+      <c r="AB21" s="6">
         <v>97</v>
       </c>
-      <c r="AC21" s="12">
+      <c r="AC21" s="6">
         <v>96.7</v>
       </c>
-      <c r="AD21" s="12">
+      <c r="AD21" s="6">
         <v>69.3</v>
       </c>
-      <c r="AE21" s="12">
+      <c r="AE21" s="6">
         <v>87.5</v>
       </c>
-      <c r="AF21" s="12">
+      <c r="AF21" s="6">
         <v>93.1</v>
       </c>
-      <c r="AG21" s="12">
+      <c r="AG21" s="6">
         <v>93.5</v>
       </c>
-      <c r="AH21" s="12">
+      <c r="AH21" s="6">
         <v>96.7</v>
       </c>
-      <c r="AI21" s="12">
+      <c r="AI21" s="6">
         <v>97.9</v>
       </c>
-      <c r="AJ21" s="12">
+      <c r="AJ21" s="6">
         <v>99.1</v>
       </c>
-      <c r="AK21" s="12">
+      <c r="AK21" s="6">
         <v>97.8</v>
       </c>
-      <c r="AL21" s="12">
+      <c r="AL21" s="6">
         <v>97</v>
       </c>
-      <c r="AM21" s="12">
+      <c r="AM21" s="6">
         <v>91.7</v>
       </c>
-      <c r="AN21" s="12">
+      <c r="AN21" s="6">
         <v>97.2</v>
       </c>
-      <c r="AO21" s="12">
+      <c r="AO21" s="6">
         <v>94.3</v>
       </c>
-      <c r="AP21" s="12">
+      <c r="AP21" s="6">
         <v>100</v>
       </c>
-      <c r="AQ21" s="12">
+      <c r="AQ21" s="6">
         <v>99.2</v>
       </c>
-      <c r="AR21" s="12">
+      <c r="AR21" s="6">
         <v>100</v>
       </c>
-      <c r="AS21" s="12">
+      <c r="AS21" s="6">
         <v>100</v>
       </c>
-      <c r="AT21" s="12">
+      <c r="AT21" s="6">
         <v>100</v>
       </c>
-      <c r="AU21" s="12">
+      <c r="AU21" s="6">
         <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -21440,141 +21435,141 @@
       <c r="C22" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="6">
         <v>49.8</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="6">
         <v>71.2</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="6">
         <v>83.6</v>
       </c>
-      <c r="G22" s="12">
+      <c r="G22" s="6">
         <v>91</v>
       </c>
-      <c r="H22" s="12">
+      <c r="H22" s="6">
         <v>93.4</v>
       </c>
-      <c r="I22" s="12">
+      <c r="I22" s="6">
         <v>93.5</v>
       </c>
-      <c r="J22" s="12">
+      <c r="J22" s="6">
         <v>91.5</v>
       </c>
-      <c r="K22" s="12">
+      <c r="K22" s="6">
         <v>91.7</v>
       </c>
       <c r="L22" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="M22" s="12">
+      <c r="M22" s="6">
         <v>40.700000000000003</v>
       </c>
-      <c r="N22" s="12">
+      <c r="N22" s="6">
         <v>61.1</v>
       </c>
-      <c r="O22" s="12">
+      <c r="O22" s="6">
         <v>81.099999999999994</v>
       </c>
-      <c r="P22" s="12">
+      <c r="P22" s="6">
         <v>89.6</v>
       </c>
-      <c r="Q22" s="12">
+      <c r="Q22" s="6">
         <v>92.8</v>
       </c>
-      <c r="R22" s="12">
+      <c r="R22" s="6">
         <v>92</v>
       </c>
-      <c r="S22" s="12">
+      <c r="S22" s="6">
         <v>89.1</v>
       </c>
-      <c r="T22" s="12">
+      <c r="T22" s="6">
         <v>90.4</v>
       </c>
       <c r="U22" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="V22" s="12">
+      <c r="V22" s="6">
         <v>85</v>
       </c>
-      <c r="W22" s="12">
+      <c r="W22" s="6">
         <v>92.3</v>
       </c>
-      <c r="X22" s="12">
+      <c r="X22" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y22" s="12">
+      <c r="Y22" s="6">
         <v>99.3</v>
       </c>
-      <c r="Z22" s="12">
+      <c r="Z22" s="6">
         <v>100</v>
       </c>
-      <c r="AA22" s="12">
+      <c r="AA22" s="6">
         <v>98</v>
       </c>
-      <c r="AB22" s="12">
+      <c r="AB22" s="6">
         <v>97</v>
       </c>
-      <c r="AC22" s="12">
+      <c r="AC22" s="6">
         <v>96.7</v>
       </c>
       <c r="AD22" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AE22" s="12">
+      <c r="AE22" s="6">
         <v>51.9</v>
       </c>
-      <c r="AF22" s="12">
+      <c r="AF22" s="6">
         <v>76.7</v>
       </c>
-      <c r="AG22" s="12">
+      <c r="AG22" s="6">
         <v>79.900000000000006</v>
       </c>
-      <c r="AH22" s="12">
+      <c r="AH22" s="6">
         <v>89.2</v>
       </c>
-      <c r="AI22" s="12">
+      <c r="AI22" s="6">
         <v>91.2</v>
       </c>
-      <c r="AJ22" s="12">
+      <c r="AJ22" s="6">
         <v>93.2</v>
       </c>
-      <c r="AK22" s="12">
+      <c r="AK22" s="6">
         <v>90.8</v>
       </c>
-      <c r="AL22" s="12">
+      <c r="AL22" s="6">
         <v>90.2</v>
       </c>
       <c r="AM22" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AN22" s="12">
+      <c r="AN22" s="6">
         <v>52.8</v>
       </c>
-      <c r="AO22" s="12">
+      <c r="AO22" s="6">
         <v>83.9</v>
       </c>
-      <c r="AP22" s="12">
+      <c r="AP22" s="6">
         <v>100</v>
       </c>
-      <c r="AQ22" s="12">
+      <c r="AQ22" s="6">
         <v>98.8</v>
       </c>
-      <c r="AR22" s="12">
+      <c r="AR22" s="6">
         <v>100</v>
       </c>
-      <c r="AS22" s="12">
+      <c r="AS22" s="6">
         <v>100</v>
       </c>
-      <c r="AT22" s="12">
+      <c r="AT22" s="6">
         <v>100</v>
       </c>
-      <c r="AU22" s="12">
+      <c r="AU22" s="6">
         <v>99.5</v>
       </c>
     </row>
     <row r="23" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B23" s="6" t="s">
@@ -21586,25 +21581,25 @@
       <c r="D23" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="6">
         <v>45.1</v>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="6">
         <v>64.099999999999994</v>
       </c>
-      <c r="G23" s="12">
+      <c r="G23" s="6">
         <v>79.599999999999994</v>
       </c>
-      <c r="H23" s="12">
+      <c r="H23" s="6">
         <v>80.8</v>
       </c>
-      <c r="I23" s="12">
+      <c r="I23" s="6">
         <v>82.6</v>
       </c>
-      <c r="J23" s="12">
+      <c r="J23" s="6">
         <v>79.5</v>
       </c>
-      <c r="K23" s="12">
+      <c r="K23" s="6">
         <v>81.7</v>
       </c>
       <c r="L23" s="6" t="s">
@@ -21613,25 +21608,25 @@
       <c r="M23" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="N23" s="12">
+      <c r="N23" s="6">
         <v>32.9</v>
       </c>
-      <c r="O23" s="12">
+      <c r="O23" s="6">
         <v>55.7</v>
       </c>
-      <c r="P23" s="12">
+      <c r="P23" s="6">
         <v>76.599999999999994</v>
       </c>
-      <c r="Q23" s="12">
+      <c r="Q23" s="6">
         <v>77.7</v>
       </c>
-      <c r="R23" s="12">
+      <c r="R23" s="6">
         <v>78.7</v>
       </c>
-      <c r="S23" s="12">
+      <c r="S23" s="6">
         <v>72.2</v>
       </c>
-      <c r="T23" s="12">
+      <c r="T23" s="6">
         <v>78.400000000000006</v>
       </c>
       <c r="U23" s="6" t="s">
@@ -21640,25 +21635,25 @@
       <c r="V23" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="W23" s="12">
+      <c r="W23" s="6">
         <v>75</v>
       </c>
-      <c r="X23" s="12">
+      <c r="X23" s="6">
         <v>98.1</v>
       </c>
-      <c r="Y23" s="12">
+      <c r="Y23" s="6">
         <v>98.6</v>
       </c>
-      <c r="Z23" s="12">
+      <c r="Z23" s="6">
         <v>100</v>
       </c>
-      <c r="AA23" s="12">
+      <c r="AA23" s="6">
         <v>97</v>
       </c>
-      <c r="AB23" s="12">
+      <c r="AB23" s="6">
         <v>96</v>
       </c>
-      <c r="AC23" s="12">
+      <c r="AC23" s="6">
         <v>95.9</v>
       </c>
       <c r="AD23" s="6" t="s">
@@ -21667,25 +21662,25 @@
       <c r="AE23" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AF23" s="12">
+      <c r="AF23" s="6">
         <v>51.3</v>
       </c>
-      <c r="AG23" s="12">
+      <c r="AG23" s="6">
         <v>62.3</v>
       </c>
-      <c r="AH23" s="12">
+      <c r="AH23" s="6">
         <v>75.599999999999994</v>
       </c>
-      <c r="AI23" s="12">
+      <c r="AI23" s="6">
         <v>76.2</v>
       </c>
-      <c r="AJ23" s="12">
+      <c r="AJ23" s="6">
         <v>81.400000000000006</v>
       </c>
-      <c r="AK23" s="12">
+      <c r="AK23" s="6">
         <v>79.8</v>
       </c>
-      <c r="AL23" s="12">
+      <c r="AL23" s="6">
         <v>78.5</v>
       </c>
       <c r="AM23" s="6" t="s">
@@ -21694,30 +21689,30 @@
       <c r="AN23" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AO23" s="12">
+      <c r="AO23" s="6">
         <v>59.8</v>
       </c>
-      <c r="AP23" s="12">
+      <c r="AP23" s="6">
         <v>89.1</v>
       </c>
-      <c r="AQ23" s="12">
+      <c r="AQ23" s="6">
         <v>96.1</v>
       </c>
-      <c r="AR23" s="12">
+      <c r="AR23" s="6">
         <v>99.5</v>
       </c>
-      <c r="AS23" s="12">
+      <c r="AS23" s="6">
         <v>98.8</v>
       </c>
-      <c r="AT23" s="12">
+      <c r="AT23" s="6">
         <v>99.1</v>
       </c>
-      <c r="AU23" s="12">
+      <c r="AU23" s="6">
         <v>97.7</v>
       </c>
     </row>
     <row r="24" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="11" t="s">
         <v>385</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -21732,22 +21727,22 @@
       <c r="E24" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="F24" s="12">
+      <c r="F24" s="6">
         <v>34</v>
       </c>
-      <c r="G24" s="12">
+      <c r="G24" s="6">
         <v>50.9</v>
       </c>
-      <c r="H24" s="12">
+      <c r="H24" s="6">
         <v>49.8</v>
       </c>
-      <c r="I24" s="12">
+      <c r="I24" s="6">
         <v>54.2</v>
       </c>
-      <c r="J24" s="12">
+      <c r="J24" s="6">
         <v>55.9</v>
       </c>
-      <c r="K24" s="12">
+      <c r="K24" s="6">
         <v>56.2</v>
       </c>
       <c r="L24" s="6" t="s">
@@ -21759,22 +21754,22 @@
       <c r="N24" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="O24" s="12">
+      <c r="O24" s="6">
         <v>25.9</v>
       </c>
-      <c r="P24" s="12">
+      <c r="P24" s="6">
         <v>35.799999999999997</v>
       </c>
-      <c r="Q24" s="12">
+      <c r="Q24" s="6">
         <v>34.700000000000003</v>
       </c>
-      <c r="R24" s="12">
+      <c r="R24" s="6">
         <v>39.1</v>
       </c>
-      <c r="S24" s="12">
+      <c r="S24" s="6">
         <v>36.6</v>
       </c>
-      <c r="T24" s="12">
+      <c r="T24" s="6">
         <v>38.9</v>
       </c>
       <c r="U24" s="6" t="s">
@@ -21786,22 +21781,22 @@
       <c r="W24" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="X24" s="12">
+      <c r="X24" s="6">
         <v>41.5</v>
       </c>
-      <c r="Y24" s="12">
+      <c r="Y24" s="6">
         <v>92.4</v>
       </c>
-      <c r="Z24" s="12">
+      <c r="Z24" s="6">
         <v>97.6</v>
       </c>
-      <c r="AA24" s="12">
+      <c r="AA24" s="6">
         <v>92.9</v>
       </c>
-      <c r="AB24" s="12">
+      <c r="AB24" s="6">
         <v>93.9</v>
       </c>
-      <c r="AC24" s="12">
+      <c r="AC24" s="6">
         <v>93.4</v>
       </c>
       <c r="AD24" s="6" t="s">
@@ -21813,22 +21808,22 @@
       <c r="AF24" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AG24" s="12">
+      <c r="AG24" s="6">
         <v>37.4</v>
       </c>
-      <c r="AH24" s="12">
+      <c r="AH24" s="6">
         <v>53</v>
       </c>
-      <c r="AI24" s="12">
+      <c r="AI24" s="6">
         <v>48.2</v>
       </c>
-      <c r="AJ24" s="12">
+      <c r="AJ24" s="6">
         <v>57.7</v>
       </c>
-      <c r="AK24" s="12">
+      <c r="AK24" s="6">
         <v>62.4</v>
       </c>
-      <c r="AL24" s="12">
+      <c r="AL24" s="6">
         <v>60.9</v>
       </c>
       <c r="AM24" s="6" t="s">
@@ -21840,85 +21835,78 @@
       <c r="AO24" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="AP24" s="12">
+      <c r="AP24" s="6">
         <v>53.5</v>
       </c>
-      <c r="AQ24" s="12">
+      <c r="AQ24" s="6">
         <v>86.4</v>
       </c>
-      <c r="AR24" s="12">
+      <c r="AR24" s="6">
         <v>97.1</v>
       </c>
-      <c r="AS24" s="12">
+      <c r="AS24" s="6">
         <v>95.8</v>
       </c>
-      <c r="AT24" s="12">
+      <c r="AT24" s="6">
         <v>94.8</v>
       </c>
-      <c r="AU24" s="12">
+      <c r="AU24" s="6">
         <v>87.9</v>
       </c>
     </row>
     <row r="26" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="12" t="s">
         <v>391</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
-      <c r="O26" s="11"/>
-      <c r="P26" s="11"/>
-      <c r="Q26" s="11"/>
-      <c r="R26" s="11"/>
-      <c r="S26" s="11"/>
-      <c r="T26" s="11"/>
-      <c r="U26" s="11"/>
-      <c r="V26" s="11"/>
-      <c r="W26" s="11"/>
-      <c r="X26" s="11"/>
-      <c r="Y26" s="11"/>
-      <c r="Z26" s="11"/>
-      <c r="AA26" s="11"/>
-      <c r="AB26" s="11"/>
-      <c r="AC26" s="11"/>
-      <c r="AD26" s="11"/>
-      <c r="AE26" s="11"/>
-      <c r="AF26" s="11"/>
-      <c r="AG26" s="11"/>
-      <c r="AH26" s="11"/>
-      <c r="AI26" s="11"/>
-      <c r="AJ26" s="11"/>
-      <c r="AK26" s="11"/>
-      <c r="AL26" s="11"/>
-      <c r="AM26" s="11"/>
-      <c r="AN26" s="11"/>
-      <c r="AO26" s="11"/>
-      <c r="AP26" s="11"/>
-      <c r="AQ26" s="11"/>
-      <c r="AR26" s="11"/>
-      <c r="AS26" s="11"/>
-      <c r="AT26" s="11"/>
-      <c r="AU26" s="11"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
+      <c r="S26" s="12"/>
+      <c r="T26" s="12"/>
+      <c r="U26" s="12"/>
+      <c r="V26" s="12"/>
+      <c r="W26" s="12"/>
+      <c r="X26" s="12"/>
+      <c r="Y26" s="12"/>
+      <c r="Z26" s="12"/>
+      <c r="AA26" s="12"/>
+      <c r="AB26" s="12"/>
+      <c r="AC26" s="12"/>
+      <c r="AD26" s="12"/>
+      <c r="AE26" s="12"/>
+      <c r="AF26" s="12"/>
+      <c r="AG26" s="12"/>
+      <c r="AH26" s="12"/>
+      <c r="AI26" s="12"/>
+      <c r="AJ26" s="12"/>
+      <c r="AK26" s="12"/>
+      <c r="AL26" s="12"/>
+      <c r="AM26" s="12"/>
+      <c r="AN26" s="12"/>
+      <c r="AO26" s="12"/>
+      <c r="AP26" s="12"/>
+      <c r="AQ26" s="12"/>
+      <c r="AR26" s="12"/>
+      <c r="AS26" s="12"/>
+      <c r="AT26" s="12"/>
+      <c r="AU26" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="A26:AU26"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A18:A20"/>
     <mergeCell ref="A1:AU1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -21927,6 +21915,13 @@
     <mergeCell ref="U2:AC2"/>
     <mergeCell ref="AD2:AL2"/>
     <mergeCell ref="AM2:AU2"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="A26:AU26"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -21938,10 +21933,10 @@
   <dimension ref="A1:E703"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.21875" customWidth="1"/>
-    <col min="2" max="2" width="18.6640625" customWidth="1"/>
+    <col min="1" max="1" width="8.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="17.21875" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
     <col min="5" max="5" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -21954,7 +21949,8 @@
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
     </row>
-    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="5.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>19</v>
       </c>
@@ -33650,7 +33646,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E3" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A3:E703" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -34842,137 +34838,132 @@
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="12" t="s">
         <v>425</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="11"/>
-      <c r="S21" s="11"/>
-      <c r="T21" s="11"/>
-      <c r="U21" s="11"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="12"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="12"/>
+      <c r="U21" s="12"/>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="12" t="s">
         <v>426</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="11"/>
-      <c r="R22" s="11"/>
-      <c r="S22" s="11"/>
-      <c r="T22" s="11"/>
-      <c r="U22" s="11"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="12"/>
+      <c r="Q22" s="12"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="12"/>
+      <c r="T22" s="12"/>
+      <c r="U22" s="12"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="11"/>
-      <c r="P23" s="11"/>
-      <c r="Q23" s="11"/>
-      <c r="R23" s="11"/>
-      <c r="S23" s="11"/>
-      <c r="T23" s="11"/>
-      <c r="U23" s="11"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="12"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="12"/>
+      <c r="T23" s="12"/>
+      <c r="U23" s="12"/>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="12" t="s">
         <v>428</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
-      <c r="R24" s="11"/>
-      <c r="S24" s="11"/>
-      <c r="T24" s="11"/>
-      <c r="U24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
+      <c r="T24" s="12"/>
+      <c r="U24" s="12"/>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
-      <c r="R25" s="11"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
-      <c r="U25" s="11"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="12"/>
+      <c r="P25" s="12"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+      <c r="S25" s="12"/>
+      <c r="T25" s="12"/>
+      <c r="U25" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A21:U21"/>
-    <mergeCell ref="A22:U22"/>
-    <mergeCell ref="A23:U23"/>
-    <mergeCell ref="A24:U24"/>
-    <mergeCell ref="A25:U25"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:C2"/>
@@ -34985,6 +34976,11 @@
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="R2:S2"/>
     <mergeCell ref="T2:U2"/>
+    <mergeCell ref="A21:U21"/>
+    <mergeCell ref="A22:U22"/>
+    <mergeCell ref="A23:U23"/>
+    <mergeCell ref="A24:U24"/>
+    <mergeCell ref="A25:U25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -34996,7 +34992,7 @@
   <dimension ref="A1:U25"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" customWidth="1"/>
     <col min="2" max="21" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -35729,267 +35725,257 @@
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="11"/>
-      <c r="S16" s="11"/>
-      <c r="T16" s="11"/>
-      <c r="U16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="12"/>
+      <c r="T16" s="12"/>
+      <c r="U16" s="12"/>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="11"/>
-      <c r="S17" s="11"/>
-      <c r="T17" s="11"/>
-      <c r="U17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="12"/>
+      <c r="U17" s="12"/>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="12" t="s">
         <v>444</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="11"/>
-      <c r="R18" s="11"/>
-      <c r="S18" s="11"/>
-      <c r="T18" s="11"/>
-      <c r="U18" s="11"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="12"/>
+      <c r="U18" s="12"/>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="12" t="s">
         <v>445</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-      <c r="S19" s="11"/>
-      <c r="T19" s="11"/>
-      <c r="U19" s="11"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+      <c r="P19" s="12"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="12"/>
+      <c r="S19" s="12"/>
+      <c r="T19" s="12"/>
+      <c r="U19" s="12"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="12" t="s">
         <v>446</v>
       </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="11"/>
-      <c r="R20" s="11"/>
-      <c r="S20" s="11"/>
-      <c r="T20" s="11"/>
-      <c r="U20" s="11"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="12"/>
+      <c r="Q20" s="12"/>
+      <c r="R20" s="12"/>
+      <c r="S20" s="12"/>
+      <c r="T20" s="12"/>
+      <c r="U20" s="12"/>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="12" t="s">
         <v>447</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="11"/>
-      <c r="S21" s="11"/>
-      <c r="T21" s="11"/>
-      <c r="U21" s="11"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="12"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="12"/>
+      <c r="U21" s="12"/>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="11"/>
-      <c r="R22" s="11"/>
-      <c r="S22" s="11"/>
-      <c r="T22" s="11"/>
-      <c r="U22" s="11"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="12"/>
+      <c r="Q22" s="12"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="12"/>
+      <c r="T22" s="12"/>
+      <c r="U22" s="12"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="12" t="s">
         <v>449</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="11"/>
-      <c r="P23" s="11"/>
-      <c r="Q23" s="11"/>
-      <c r="R23" s="11"/>
-      <c r="S23" s="11"/>
-      <c r="T23" s="11"/>
-      <c r="U23" s="11"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="12"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="12"/>
+      <c r="T23" s="12"/>
+      <c r="U23" s="12"/>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="12" t="s">
         <v>450</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
-      <c r="R24" s="11"/>
-      <c r="S24" s="11"/>
-      <c r="T24" s="11"/>
-      <c r="U24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
+      <c r="T24" s="12"/>
+      <c r="U24" s="12"/>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="12" t="s">
         <v>451</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
-      <c r="R25" s="11"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
-      <c r="U25" s="11"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="12"/>
+      <c r="P25" s="12"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+      <c r="S25" s="12"/>
+      <c r="T25" s="12"/>
+      <c r="U25" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A21:U21"/>
-    <mergeCell ref="A22:U22"/>
-    <mergeCell ref="A23:U23"/>
-    <mergeCell ref="A24:U24"/>
-    <mergeCell ref="A25:U25"/>
-    <mergeCell ref="A16:U16"/>
-    <mergeCell ref="A17:U17"/>
-    <mergeCell ref="A18:U18"/>
-    <mergeCell ref="A19:U19"/>
-    <mergeCell ref="A20:U20"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:C2"/>
@@ -36002,6 +35988,16 @@
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="R2:S2"/>
     <mergeCell ref="T2:U2"/>
+    <mergeCell ref="A16:U16"/>
+    <mergeCell ref="A17:U17"/>
+    <mergeCell ref="A18:U18"/>
+    <mergeCell ref="A19:U19"/>
+    <mergeCell ref="A20:U20"/>
+    <mergeCell ref="A21:U21"/>
+    <mergeCell ref="A22:U22"/>
+    <mergeCell ref="A23:U23"/>
+    <mergeCell ref="A24:U24"/>
+    <mergeCell ref="A25:U25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>